<commit_message>
runs PFOA model humans
</commit_message>
<xml_diff>
--- a/PFOA extrapolation to humans/Data/Abraham et al.2024_oral_feces_cut.xlsx
+++ b/PFOA extrapolation to humans/Data/Abraham et al.2024_oral_feces_cut.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eviepapakyriakopoulou/Documents/Documents/NTUA Post-Doc/CHIASMA/PFOA extrapolation humans/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eviepapakyriakopoulou/Documents/GitHub/PFAS_PBK_models/PFOA extrapolation to humans/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72FE5EAE-9FA0-7C46-99E2-9CB954A27DAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82E38D37-1012-7447-820F-5574E804C494}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1040" yWindow="680" windowWidth="28360" windowHeight="18440" xr2:uid="{3744AC73-CAAE-7E42-A2FB-1EDC36DFABA9}"/>
+    <workbookView xWindow="420" yWindow="-19480" windowWidth="28340" windowHeight="18440" xr2:uid="{3744AC73-CAAE-7E42-A2FB-1EDC36DFABA9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -75,11 +75,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -107,12 +108,6 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -134,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -146,9 +141,6 @@
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -158,10 +150,10 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -498,18 +490,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79597772-21D1-314A-89B1-40D073D89A86}">
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="3"/>
     <col min="2" max="2" width="12.6640625" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="12.6640625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="19.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.33203125" style="3" customWidth="1"/>
     <col min="6" max="6" width="13.83203125" style="3" bestFit="1" customWidth="1"/>
     <col min="7" max="16384" width="10.83203125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -535,28 +527,27 @@
         <v>7</v>
       </c>
       <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
       <c r="K1" s="2"/>
       <c r="L1" s="2"/>
     </row>
-    <row r="2" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="7">
-        <v>60</v>
-      </c>
-      <c r="C2" s="8">
+      <c r="B2" s="6">
+        <v>24</v>
+      </c>
+      <c r="C2" s="7">
         <f>D2*E2</f>
         <v>0.6115149240364145</v>
       </c>
-      <c r="D2" s="7">
+      <c r="D2" s="2">
         <v>260</v>
       </c>
       <c r="E2" s="9">
         <v>2.3519804770631325E-3</v>
       </c>
-      <c r="F2" s="6">
+      <c r="F2" s="5">
         <f>3.96*0.04/100</f>
         <v>1.5840000000000001E-3</v>
       </c>
@@ -567,28 +558,27 @@
         <v>10</v>
       </c>
       <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
       <c r="K2" s="4"/>
       <c r="L2" s="2"/>
     </row>
-    <row r="3" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="7">
-        <v>120</v>
-      </c>
-      <c r="C3" s="8">
+      <c r="B3" s="6">
+        <v>48</v>
+      </c>
+      <c r="C3" s="7">
         <f t="shared" ref="C3:C7" si="0">D3*E3</f>
         <v>0.60388741183260231</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="2">
         <v>162</v>
       </c>
       <c r="E3" s="9">
         <v>3.7277000730407549E-3</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F3" s="5">
         <v>1.5840000000000001E-3</v>
       </c>
       <c r="G3" s="2" t="s">
@@ -597,29 +587,28 @@
       <c r="H3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="10"/>
-      <c r="J3" s="2"/>
+      <c r="I3" s="2"/>
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
     </row>
-    <row r="4" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="7">
-        <v>180</v>
-      </c>
-      <c r="C4" s="8">
+      <c r="B4" s="6">
+        <v>72</v>
+      </c>
+      <c r="C4" s="7">
         <f t="shared" si="0"/>
         <v>0.47049627352340628</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="2">
         <v>328</v>
       </c>
       <c r="E4" s="9">
         <v>1.434439858303068E-3</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="5">
         <v>1.5840000000000001E-3</v>
       </c>
       <c r="G4" s="2" t="s">
@@ -629,26 +618,26 @@
         <v>10</v>
       </c>
       <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
+      <c r="L4" s="2"/>
     </row>
-    <row r="5" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="7">
-        <v>240</v>
-      </c>
-      <c r="C5" s="8">
+      <c r="B5" s="6">
+        <v>96</v>
+      </c>
+      <c r="C5" s="7">
         <f t="shared" si="0"/>
         <v>0.51750168663250129</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="2">
         <v>202</v>
       </c>
       <c r="E5" s="9">
         <v>2.5618895377846596E-3</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="5">
         <v>1.5840000000000001E-3</v>
       </c>
       <c r="G5" s="2" t="s">
@@ -658,25 +647,26 @@
         <v>10</v>
       </c>
       <c r="I5" s="2"/>
+      <c r="L5" s="2"/>
     </row>
-    <row r="6" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="7">
-        <v>300</v>
-      </c>
-      <c r="C6" s="8">
+      <c r="B6" s="6">
+        <v>120</v>
+      </c>
+      <c r="C6" s="7">
         <f t="shared" si="0"/>
         <v>0.6680692063407031</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="2">
         <v>248</v>
       </c>
       <c r="E6" s="9">
         <v>2.69382744492219E-3</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="5">
         <v>1.5840000000000001E-3</v>
       </c>
       <c r="G6" s="2" t="s">
@@ -686,25 +676,30 @@
         <v>10</v>
       </c>
       <c r="I6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="6"/>
+      <c r="N6" s="7"/>
+      <c r="O6" s="6"/>
+      <c r="P6" s="8"/>
     </row>
-    <row r="7" spans="1:12" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="7">
-        <v>360</v>
-      </c>
-      <c r="C7" s="8">
+      <c r="B7" s="6">
+        <v>144</v>
+      </c>
+      <c r="C7" s="7">
         <f t="shared" si="0"/>
         <v>0.4149654833040059</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="2">
         <v>90</v>
       </c>
       <c r="E7" s="9">
         <v>4.6107275922667324E-3</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="5">
         <v>1.5840000000000001E-3</v>
       </c>
       <c r="G7" s="2" t="s">
@@ -714,79 +709,11 @@
         <v>10</v>
       </c>
       <c r="I7" s="2"/>
-    </row>
-    <row r="8" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="B8" s="7"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-    </row>
-    <row r="9" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="B9" s="7"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-    </row>
-    <row r="10" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="B10" s="7"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="5"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-    </row>
-    <row r="11" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="B11" s="7"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-    </row>
-    <row r="12" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="B12" s="7"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="5"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-    </row>
-    <row r="13" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="B13" s="7"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="5"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-    </row>
-    <row r="14" spans="1:12" ht="16" x14ac:dyDescent="0.2">
-      <c r="B14" s="7"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="H15" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="6"/>
+      <c r="N7" s="7"/>
+      <c r="O7" s="6"/>
+      <c r="P7" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>